<commit_message>
fix(qc): correct ANNEXE F data validations to Statut column G
Replace the audit gabarit so Fiche modèle has a single status list on G17:G89 (73 cells), removing the shifted list on F and Oui/Non on G.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/backend/templates/ANNEXE_F_-_Checklist_CQ_BIM.xlsx
+++ b/backend/templates/ANNEXE_F_-_Checklist_CQ_BIM.xlsx
@@ -203,7 +203,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -284,11 +284,55 @@
         <color rgb="FFB0B0B0"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFB0B0B0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFB0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB0B0B0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFB0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFB0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -388,6 +432,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1142,13 +1188,13 @@
           <t>1. Fichier</t>
         </is>
       </c>
-      <c r="B4" s="27" t="n"/>
-      <c r="C4" s="27" t="n"/>
-      <c r="D4" s="27" t="n"/>
-      <c r="E4" s="27" t="n"/>
-      <c r="F4" s="27" t="n"/>
-      <c r="G4" s="27" t="n"/>
-      <c r="H4" s="27" t="n"/>
+      <c r="B4" s="37" t="n"/>
+      <c r="C4" s="37" t="n"/>
+      <c r="D4" s="37" t="n"/>
+      <c r="E4" s="37" t="n"/>
+      <c r="F4" s="37" t="n"/>
+      <c r="G4" s="37" t="n"/>
+      <c r="H4" s="38" t="n"/>
     </row>
     <row r="5" ht="22.8" customHeight="1" s="11">
       <c r="A5" s="28" t="inlineStr">
@@ -1644,13 +1690,13 @@
           <t>2. Positionnement</t>
         </is>
       </c>
-      <c r="B17" s="27" t="n"/>
-      <c r="C17" s="27" t="n"/>
-      <c r="D17" s="27" t="n"/>
-      <c r="E17" s="27" t="n"/>
-      <c r="F17" s="27" t="n"/>
-      <c r="G17" s="27" t="n"/>
-      <c r="H17" s="27" t="n"/>
+      <c r="B17" s="37" t="n"/>
+      <c r="C17" s="37" t="n"/>
+      <c r="D17" s="37" t="n"/>
+      <c r="E17" s="37" t="n"/>
+      <c r="F17" s="37" t="n"/>
+      <c r="G17" s="37" t="n"/>
+      <c r="H17" s="38" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="28" t="inlineStr">
@@ -2062,13 +2108,13 @@
           <t>3. Contenu de la modélisation</t>
         </is>
       </c>
-      <c r="B28" s="27" t="n"/>
-      <c r="C28" s="27" t="n"/>
-      <c r="D28" s="27" t="n"/>
-      <c r="E28" s="27" t="n"/>
-      <c r="F28" s="27" t="n"/>
-      <c r="G28" s="27" t="n"/>
-      <c r="H28" s="27" t="n"/>
+      <c r="B28" s="37" t="n"/>
+      <c r="C28" s="37" t="n"/>
+      <c r="D28" s="37" t="n"/>
+      <c r="E28" s="37" t="n"/>
+      <c r="F28" s="37" t="n"/>
+      <c r="G28" s="37" t="n"/>
+      <c r="H28" s="38" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="28" t="inlineStr">
@@ -2578,13 +2624,13 @@
           <t>4. Organisation Revit</t>
         </is>
       </c>
-      <c r="B42" s="27" t="n"/>
-      <c r="C42" s="27" t="n"/>
-      <c r="D42" s="27" t="n"/>
-      <c r="E42" s="27" t="n"/>
-      <c r="F42" s="27" t="n"/>
-      <c r="G42" s="27" t="n"/>
-      <c r="H42" s="27" t="n"/>
+      <c r="B42" s="37" t="n"/>
+      <c r="C42" s="37" t="n"/>
+      <c r="D42" s="37" t="n"/>
+      <c r="E42" s="37" t="n"/>
+      <c r="F42" s="37" t="n"/>
+      <c r="G42" s="37" t="n"/>
+      <c r="H42" s="38" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="28" t="inlineStr">
@@ -3080,13 +3126,13 @@
           <t>5. Paramètres</t>
         </is>
       </c>
-      <c r="B55" s="27" t="n"/>
-      <c r="C55" s="27" t="n"/>
-      <c r="D55" s="27" t="n"/>
-      <c r="E55" s="27" t="n"/>
-      <c r="F55" s="27" t="n"/>
-      <c r="G55" s="27" t="n"/>
-      <c r="H55" s="27" t="n"/>
+      <c r="B55" s="37" t="n"/>
+      <c r="C55" s="37" t="n"/>
+      <c r="D55" s="37" t="n"/>
+      <c r="E55" s="37" t="n"/>
+      <c r="F55" s="37" t="n"/>
+      <c r="G55" s="37" t="n"/>
+      <c r="H55" s="38" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="28" t="inlineStr">
@@ -3528,13 +3574,13 @@
           <t>6. Export et métadonnées</t>
         </is>
       </c>
-      <c r="B67" s="27" t="n"/>
-      <c r="C67" s="27" t="n"/>
-      <c r="D67" s="27" t="n"/>
-      <c r="E67" s="27" t="n"/>
-      <c r="F67" s="27" t="n"/>
-      <c r="G67" s="27" t="n"/>
-      <c r="H67" s="27" t="n"/>
+      <c r="B67" s="37" t="n"/>
+      <c r="C67" s="37" t="n"/>
+      <c r="D67" s="37" t="n"/>
+      <c r="E67" s="37" t="n"/>
+      <c r="F67" s="37" t="n"/>
+      <c r="G67" s="37" t="n"/>
+      <c r="H67" s="38" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="28" t="inlineStr">
@@ -4150,13 +4196,13 @@
           <t>1. Fichier</t>
         </is>
       </c>
-      <c r="B17" s="27" t="n"/>
-      <c r="C17" s="27" t="n"/>
-      <c r="D17" s="27" t="n"/>
-      <c r="E17" s="27" t="n"/>
-      <c r="F17" s="27" t="n"/>
-      <c r="G17" s="27" t="n"/>
-      <c r="H17" s="27" t="n"/>
+      <c r="B17" s="37" t="n"/>
+      <c r="C17" s="37" t="n"/>
+      <c r="D17" s="37" t="n"/>
+      <c r="E17" s="37" t="n"/>
+      <c r="F17" s="37" t="n"/>
+      <c r="G17" s="37" t="n"/>
+      <c r="H17" s="38" t="n"/>
     </row>
     <row r="18" ht="22.8" customHeight="1" s="11">
       <c r="A18" s="28" t="inlineStr">
@@ -4524,13 +4570,13 @@
           <t>2. Positionnement</t>
         </is>
       </c>
-      <c r="B30" s="27" t="n"/>
-      <c r="C30" s="27" t="n"/>
-      <c r="D30" s="27" t="n"/>
-      <c r="E30" s="27" t="n"/>
-      <c r="F30" s="27" t="n"/>
-      <c r="G30" s="27" t="n"/>
-      <c r="H30" s="27" t="n"/>
+      <c r="B30" s="37" t="n"/>
+      <c r="C30" s="37" t="n"/>
+      <c r="D30" s="37" t="n"/>
+      <c r="E30" s="37" t="n"/>
+      <c r="F30" s="37" t="n"/>
+      <c r="G30" s="37" t="n"/>
+      <c r="H30" s="38" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="28" t="inlineStr">
@@ -4838,13 +4884,13 @@
           <t>3. Contenu de la modélisation</t>
         </is>
       </c>
-      <c r="B41" s="27" t="n"/>
-      <c r="C41" s="27" t="n"/>
-      <c r="D41" s="27" t="n"/>
-      <c r="E41" s="27" t="n"/>
-      <c r="F41" s="27" t="n"/>
-      <c r="G41" s="27" t="n"/>
-      <c r="H41" s="27" t="n"/>
+      <c r="B41" s="37" t="n"/>
+      <c r="C41" s="37" t="n"/>
+      <c r="D41" s="37" t="n"/>
+      <c r="E41" s="37" t="n"/>
+      <c r="F41" s="37" t="n"/>
+      <c r="G41" s="37" t="n"/>
+      <c r="H41" s="38" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="28" t="inlineStr">
@@ -5242,13 +5288,13 @@
           <t>4. Organisation Revit</t>
         </is>
       </c>
-      <c r="B55" s="27" t="n"/>
-      <c r="C55" s="27" t="n"/>
-      <c r="D55" s="27" t="n"/>
-      <c r="E55" s="27" t="n"/>
-      <c r="F55" s="27" t="n"/>
-      <c r="G55" s="27" t="n"/>
-      <c r="H55" s="27" t="n"/>
+      <c r="B55" s="37" t="n"/>
+      <c r="C55" s="37" t="n"/>
+      <c r="D55" s="37" t="n"/>
+      <c r="E55" s="37" t="n"/>
+      <c r="F55" s="37" t="n"/>
+      <c r="G55" s="37" t="n"/>
+      <c r="H55" s="38" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="28" t="inlineStr">
@@ -5616,13 +5662,13 @@
           <t>5. Paramètres</t>
         </is>
       </c>
-      <c r="B68" s="27" t="n"/>
-      <c r="C68" s="27" t="n"/>
-      <c r="D68" s="27" t="n"/>
-      <c r="E68" s="27" t="n"/>
-      <c r="F68" s="27" t="n"/>
-      <c r="G68" s="27" t="n"/>
-      <c r="H68" s="27" t="n"/>
+      <c r="B68" s="37" t="n"/>
+      <c r="C68" s="37" t="n"/>
+      <c r="D68" s="37" t="n"/>
+      <c r="E68" s="37" t="n"/>
+      <c r="F68" s="37" t="n"/>
+      <c r="G68" s="37" t="n"/>
+      <c r="H68" s="38" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="28" t="inlineStr">
@@ -5960,13 +6006,13 @@
           <t>6. Export et métadonnées</t>
         </is>
       </c>
-      <c r="B80" s="27" t="n"/>
-      <c r="C80" s="27" t="n"/>
-      <c r="D80" s="27" t="n"/>
-      <c r="E80" s="27" t="n"/>
-      <c r="F80" s="27" t="n"/>
-      <c r="G80" s="27" t="n"/>
-      <c r="H80" s="27" t="n"/>
+      <c r="B80" s="37" t="n"/>
+      <c r="C80" s="37" t="n"/>
+      <c r="D80" s="37" t="n"/>
+      <c r="E80" s="37" t="n"/>
+      <c r="F80" s="37" t="n"/>
+      <c r="G80" s="37" t="n"/>
+      <c r="H80" s="38" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="28" t="inlineStr">
@@ -6296,12 +6342,9 @@
       <formula>"Oui"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
-    <dataValidation sqref="F17:F89" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+  <dataValidations count="1">
+    <dataValidation sqref="G17:G89" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Statut invalide" error="Choisir un statut dans la liste." promptTitle="Statut du point de contrôle" prompt="OK, À réviser, À compléter, N.A. ou Contrôle à venir" type="list">
       <formula1>"OK,À réviser,À compléter,N.A.,Contrôle à venir"</formula1>
-    </dataValidation>
-    <dataValidation sqref="G17:G89" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Oui,Non"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
@@ -6388,15 +6431,15 @@
           <t>1. Fichier</t>
         </is>
       </c>
-      <c r="B3" s="27" t="n"/>
-      <c r="C3" s="27" t="n"/>
-      <c r="D3" s="27" t="n"/>
-      <c r="E3" s="27" t="n"/>
-      <c r="F3" s="27" t="n"/>
-      <c r="G3" s="27" t="n"/>
-      <c r="H3" s="27" t="n"/>
-      <c r="I3" s="27" t="n"/>
-      <c r="J3" s="27" t="n"/>
+      <c r="B3" s="37" t="n"/>
+      <c r="C3" s="37" t="n"/>
+      <c r="D3" s="37" t="n"/>
+      <c r="E3" s="37" t="n"/>
+      <c r="F3" s="37" t="n"/>
+      <c r="G3" s="37" t="n"/>
+      <c r="H3" s="37" t="n"/>
+      <c r="I3" s="37" t="n"/>
+      <c r="J3" s="38" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="28" t="inlineStr">
@@ -6644,15 +6687,15 @@
           <t>2. Positionnement</t>
         </is>
       </c>
-      <c r="B16" s="27" t="n"/>
-      <c r="C16" s="27" t="n"/>
-      <c r="D16" s="27" t="n"/>
-      <c r="E16" s="27" t="n"/>
-      <c r="F16" s="27" t="n"/>
-      <c r="G16" s="27" t="n"/>
-      <c r="H16" s="27" t="n"/>
-      <c r="I16" s="27" t="n"/>
-      <c r="J16" s="27" t="n"/>
+      <c r="B16" s="37" t="n"/>
+      <c r="C16" s="37" t="n"/>
+      <c r="D16" s="37" t="n"/>
+      <c r="E16" s="37" t="n"/>
+      <c r="F16" s="37" t="n"/>
+      <c r="G16" s="37" t="n"/>
+      <c r="H16" s="37" t="n"/>
+      <c r="I16" s="37" t="n"/>
+      <c r="J16" s="38" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="28" t="inlineStr">
@@ -6860,15 +6903,15 @@
           <t>3. Contenu de la modélisation</t>
         </is>
       </c>
-      <c r="B27" s="27" t="n"/>
-      <c r="C27" s="27" t="n"/>
-      <c r="D27" s="27" t="n"/>
-      <c r="E27" s="27" t="n"/>
-      <c r="F27" s="27" t="n"/>
-      <c r="G27" s="27" t="n"/>
-      <c r="H27" s="27" t="n"/>
-      <c r="I27" s="27" t="n"/>
-      <c r="J27" s="27" t="n"/>
+      <c r="B27" s="37" t="n"/>
+      <c r="C27" s="37" t="n"/>
+      <c r="D27" s="37" t="n"/>
+      <c r="E27" s="37" t="n"/>
+      <c r="F27" s="37" t="n"/>
+      <c r="G27" s="37" t="n"/>
+      <c r="H27" s="37" t="n"/>
+      <c r="I27" s="37" t="n"/>
+      <c r="J27" s="38" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="28" t="inlineStr">
@@ -7136,15 +7179,15 @@
           <t>4. Organisation Revit</t>
         </is>
       </c>
-      <c r="B41" s="27" t="n"/>
-      <c r="C41" s="27" t="n"/>
-      <c r="D41" s="27" t="n"/>
-      <c r="E41" s="27" t="n"/>
-      <c r="F41" s="27" t="n"/>
-      <c r="G41" s="27" t="n"/>
-      <c r="H41" s="27" t="n"/>
-      <c r="I41" s="27" t="n"/>
-      <c r="J41" s="27" t="n"/>
+      <c r="B41" s="37" t="n"/>
+      <c r="C41" s="37" t="n"/>
+      <c r="D41" s="37" t="n"/>
+      <c r="E41" s="37" t="n"/>
+      <c r="F41" s="37" t="n"/>
+      <c r="G41" s="37" t="n"/>
+      <c r="H41" s="37" t="n"/>
+      <c r="I41" s="37" t="n"/>
+      <c r="J41" s="38" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="28" t="inlineStr">
@@ -7392,15 +7435,15 @@
           <t>5. Paramètres</t>
         </is>
       </c>
-      <c r="B54" s="27" t="n"/>
-      <c r="C54" s="27" t="n"/>
-      <c r="D54" s="27" t="n"/>
-      <c r="E54" s="27" t="n"/>
-      <c r="F54" s="27" t="n"/>
-      <c r="G54" s="27" t="n"/>
-      <c r="H54" s="27" t="n"/>
-      <c r="I54" s="27" t="n"/>
-      <c r="J54" s="27" t="n"/>
+      <c r="B54" s="37" t="n"/>
+      <c r="C54" s="37" t="n"/>
+      <c r="D54" s="37" t="n"/>
+      <c r="E54" s="37" t="n"/>
+      <c r="F54" s="37" t="n"/>
+      <c r="G54" s="37" t="n"/>
+      <c r="H54" s="37" t="n"/>
+      <c r="I54" s="37" t="n"/>
+      <c r="J54" s="38" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="28" t="inlineStr">
@@ -7628,15 +7671,15 @@
           <t>6. Export et métadonnées</t>
         </is>
       </c>
-      <c r="B66" s="27" t="n"/>
-      <c r="C66" s="27" t="n"/>
-      <c r="D66" s="27" t="n"/>
-      <c r="E66" s="27" t="n"/>
-      <c r="F66" s="27" t="n"/>
-      <c r="G66" s="27" t="n"/>
-      <c r="H66" s="27" t="n"/>
-      <c r="I66" s="27" t="n"/>
-      <c r="J66" s="27" t="n"/>
+      <c r="B66" s="37" t="n"/>
+      <c r="C66" s="37" t="n"/>
+      <c r="D66" s="37" t="n"/>
+      <c r="E66" s="37" t="n"/>
+      <c r="F66" s="37" t="n"/>
+      <c r="G66" s="37" t="n"/>
+      <c r="H66" s="37" t="n"/>
+      <c r="I66" s="37" t="n"/>
+      <c r="J66" s="38" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="28" t="inlineStr">

</xml_diff>